<commit_message>
proyectos-redaccion y metricas cna
</commit_message>
<xml_diff>
--- a/data/raw/Proyectos/centroDeProyectos_PMO_2026.xlsx
+++ b/data/raw/Proyectos/centroDeProyectos_PMO_2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5f15395a9ed9a48f/Proyectos_DS/SGING/data/raw/Proyectos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="66" documentId="11_C027D363B901AF65D94FC13C36333C815A25773C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A176856A-6B8A-4BE7-BC8A-8B7B46131741}"/>
+  <xr:revisionPtr revIDLastSave="67" documentId="11_C027D363B901AF65D94FC13C36333C815A25773C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C101444B-2D23-4103-94DA-39C6D92F1046}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2328,7 +2328,7 @@
     <col min="18" max="18" width="23" customWidth="1"/>
     <col min="19" max="19" width="11.109375" customWidth="1"/>
     <col min="21" max="22" width="26.5546875" customWidth="1"/>
-    <col min="23" max="23" width="39.109375" customWidth="1"/>
+    <col min="23" max="23" width="84.5546875" customWidth="1"/>
     <col min="24" max="26" width="55" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>